<commit_message>
Give the app its own lane in the boss summary, with store review time.
The timeline now has an App lane: accounts and the bridge plan (W1–W2),
shell and brand pages (W3–W6), a test build (W7), store review with room
for one rejection (W8–W9, submitted 11/30), client acceptance and public
release. M3 now requires installable test builds of all three apps and
open developer accounts; M4 notes the 11/30 submission.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/項目里程碑與驗收標準.xlsx
+++ b/docs/項目里程碑與驗收標準.xlsx
@@ -82,7 +82,7 @@
       <sz val="10.5"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -102,6 +102,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E0E8F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFE3F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -208,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -231,10 +236,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -242,7 +250,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -622,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -843,7 +851,7 @@
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>軟件（系統＋三個 App）</t>
+          <t>系統（三個品牌的後台）</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -860,7 +868,7 @@
       <c r="H9" s="10" t="n"/>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>送審、系統上線</t>
+          <t>三套系統上線</t>
         </is>
       </c>
       <c r="J9" s="10" t="n"/>
@@ -877,124 +885,166 @@
       </c>
       <c r="Q9" s="10" t="n"/>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>App（網頁＋原生殼）</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>開帳號、對接方案</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>殼開發、品牌頁面</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>測試版</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>商店審核</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="n"/>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>客戶驗收</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="n"/>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>公開上架</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>◆ M1</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>◆ M2</t>
         </is>
       </c>
-      <c r="H10" s="13" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>◆ M3</t>
         </is>
       </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>◆ M4</t>
         </is>
       </c>
-      <c r="M10" s="13" t="inlineStr">
+      <c r="M11" s="14" t="inlineStr">
         <is>
           <t>◆ M5</t>
         </is>
       </c>
-      <c r="O10" s="13" t="inlineStr">
+      <c r="O11" s="14" t="inlineStr">
         <is>
           <t>◆ M6</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q11" s="14" t="inlineStr">
         <is>
           <t>◆ M7</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>W11、W12 有聖誕和元旦假期；W13 留作緩衝週。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>W11、W12 有聖誕和元旦假期；W13 留作緩衝週。App 在 11/30 提交審核，預留兩週給審核和被拒後重交，趕在聖誕審核放慢之前通過。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>二、里程碑和驗收標準</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>里程碑／日期</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="16" t="n"/>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>要做到什麼</t>
         </is>
       </c>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="15" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="14" t="inlineStr">
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="16" t="n"/>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="15" t="inlineStr">
         <is>
           <t>驗收標準（全部做到才算完成）</t>
         </is>
       </c>
-      <c r="J14" s="15" t="n"/>
-      <c r="K14" s="15" t="n"/>
-      <c r="L14" s="15" t="n"/>
-      <c r="M14" s="15" t="n"/>
-      <c r="N14" s="15" t="n"/>
-      <c r="O14" s="16" t="n"/>
-      <c r="P14" s="14" t="inlineStr">
+      <c r="J15" s="16" t="n"/>
+      <c r="K15" s="16" t="n"/>
+      <c r="L15" s="16" t="n"/>
+      <c r="M15" s="16" t="n"/>
+      <c r="N15" s="16" t="n"/>
+      <c r="O15" s="17" t="n"/>
+      <c r="P15" s="15" t="inlineStr">
         <is>
           <t>誰負責</t>
         </is>
       </c>
-      <c r="Q14" s="16" t="n"/>
-    </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="Q15" s="17" t="n"/>
+    </row>
+    <row r="16" ht="95" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>M1
 10/30（五）</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>方案定案</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n"/>
-      <c r="D15" s="16" t="n"/>
-      <c r="E15" s="19" t="inlineStr">
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>量產電路板定案；第一版公仔樣品完成實測；內部測試準備好</t>
         </is>
       </c>
-      <c r="F15" s="15" t="n"/>
-      <c r="G15" s="15" t="n"/>
-      <c r="H15" s="16" t="n"/>
-      <c r="I15" s="19" t="inlineStr">
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="20" t="inlineStr">
         <is>
           <t>① 電路板連續對話 2 小時不當機、不重啟
 ② 安全加密在測試板上驗證可行
@@ -1002,43 +1052,43 @@
 ④ 20 台內部測試機準備好</t>
         </is>
       </c>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="15" t="n"/>
-      <c r="L15" s="15" t="n"/>
-      <c r="M15" s="15" t="n"/>
-      <c r="N15" s="15" t="n"/>
-      <c r="O15" s="16" t="n"/>
-      <c r="P15" s="20" t="inlineStr">
+      <c r="J16" s="16" t="n"/>
+      <c r="K16" s="16" t="n"/>
+      <c r="L16" s="16" t="n"/>
+      <c r="M16" s="16" t="n"/>
+      <c r="N16" s="16" t="n"/>
+      <c r="O16" s="17" t="n"/>
+      <c r="P16" s="21" t="inlineStr">
         <is>
           <t>我方
 玩具廠</t>
         </is>
       </c>
-      <c r="Q15" s="16" t="n"/>
-    </row>
-    <row r="16" ht="112" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="Q16" s="17" t="n"/>
+    </row>
+    <row r="17" ht="112" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>M2
 11/13（五）</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>外觀定稿、電路板下單</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="16" t="n"/>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>客戶確認公仔外觀；機芯盒開模；量產電路板下單</t>
         </is>
       </c>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="15" t="n"/>
-      <c r="H16" s="16" t="n"/>
-      <c r="I16" s="19" t="inlineStr">
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="16" t="n"/>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="20" t="inlineStr">
         <is>
           <t>① 馬會（兩款）和政協青年聯會版的外觀，由客戶書面簽樣
 ② 機芯盒設計定稿並已開模
@@ -1046,175 +1096,176 @@
 ④ 出廠韌體的底層部分（分區、加密）凍結</t>
         </is>
       </c>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="15" t="n"/>
-      <c r="L16" s="15" t="n"/>
-      <c r="M16" s="15" t="n"/>
-      <c r="N16" s="15" t="n"/>
-      <c r="O16" s="16" t="n"/>
-      <c r="P16" s="20" t="inlineStr">
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="16" t="n"/>
+      <c r="L17" s="16" t="n"/>
+      <c r="M17" s="16" t="n"/>
+      <c r="N17" s="16" t="n"/>
+      <c r="O17" s="17" t="n"/>
+      <c r="P17" s="21" t="inlineStr">
         <is>
           <t>客戶
 玩具廠
 我方</t>
         </is>
       </c>
-      <c r="Q16" s="16" t="n"/>
-    </row>
-    <row r="17" ht="146" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="Q17" s="17" t="n"/>
+    </row>
+    <row r="18" ht="197" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>M3
 11/27（五）</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B18" s="19" t="inlineStr">
         <is>
           <t>產前樣確認、大貨下單</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="16" t="n"/>
-      <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>確認產前樣，正式下大貨單；內部測試完成</t>
-        </is>
-      </c>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="16" t="n"/>
-      <c r="I17" s="19" t="inlineStr">
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>確認產前樣，正式下大貨單；內部測試完成；App 測試版完成</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="n"/>
+      <c r="G18" s="16" t="n"/>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="20" t="inlineStr">
         <is>
           <t>① 產前樣雙方簽字
 ② 大貨單已發出：馬會 2,500（兩款各多少，馬會 11/20 前確定）、政協青年聯會 500；AI Buddy 是否出貨、數量在此定案
 ③ 內部測試 4 週報告：對話穩定、回應速度達標、沒有不當內容
-④ 出廠韌體定版，交電路板廠燒錄</t>
-        </is>
-      </c>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="15" t="n"/>
-      <c r="M17" s="15" t="n"/>
-      <c r="N17" s="15" t="n"/>
-      <c r="O17" s="16" t="n"/>
-      <c r="P17" s="20" t="inlineStr">
+④ 出廠韌體定版，交電路板廠燒錄
+⑤ 三個 App 測試版可以安裝使用（藍牙配網、登入、對話）；馬會和政協青年聯會的開發者帳號已開通</t>
+        </is>
+      </c>
+      <c r="J18" s="16" t="n"/>
+      <c r="K18" s="16" t="n"/>
+      <c r="L18" s="16" t="n"/>
+      <c r="M18" s="16" t="n"/>
+      <c r="N18" s="16" t="n"/>
+      <c r="O18" s="17" t="n"/>
+      <c r="P18" s="21" t="inlineStr">
         <is>
           <t>我方
 玩具廠
 客戶</t>
         </is>
       </c>
-      <c r="Q17" s="16" t="n"/>
-    </row>
-    <row r="18" ht="112" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="Q18" s="17" t="n"/>
+    </row>
+    <row r="19" ht="112" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>M4
 12/11（五）</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>試產通過、App 過審</t>
         </is>
       </c>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="16" t="n"/>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>試產合格；三個 App 通過蘋果和 Google 審核；三個品牌的系統上線</t>
         </is>
       </c>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="15" t="n"/>
-      <c r="H18" s="16" t="n"/>
-      <c r="I18" s="19" t="inlineStr">
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="17" t="n"/>
+      <c r="I19" s="20" t="inlineStr">
         <is>
           <t>① 試產 50–100 隻全數檢查合格，發現的問題已改好
-② 三個 App 都通過蘋果和 Google 審核
+② 三個 App 都通過蘋果和 Google 審核（11/30 提交）
 ③ 玩具安全、無線、電池的檢測報告合格
 ④ 三個品牌各自的系統上線，測試全部通過</t>
         </is>
       </c>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="15" t="n"/>
-      <c r="M18" s="15" t="n"/>
-      <c r="N18" s="15" t="n"/>
-      <c r="O18" s="16" t="n"/>
-      <c r="P18" s="20" t="inlineStr">
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="16" t="n"/>
+      <c r="M19" s="16" t="n"/>
+      <c r="N19" s="16" t="n"/>
+      <c r="O19" s="17" t="n"/>
+      <c r="P19" s="21" t="inlineStr">
         <is>
           <t>玩具廠
 我方
 客戶</t>
         </is>
       </c>
-      <c r="Q18" s="16" t="n"/>
-    </row>
-    <row r="19" ht="61" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="Q19" s="17" t="n"/>
+    </row>
+    <row r="20" ht="61" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>M5
 12/31（四）</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>大貨完成</t>
         </is>
       </c>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>全部大貨生產完成</t>
         </is>
       </c>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="16" t="n"/>
-      <c r="I19" s="19" t="inlineStr">
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="17" t="n"/>
+      <c r="I20" s="20" t="inlineStr">
         <is>
           <t>① 3,000 隻（及 AI Buddy 數量）生產完成
 ② 中期驗貨抽檢合格</t>
         </is>
       </c>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="15" t="n"/>
-      <c r="M19" s="15" t="n"/>
-      <c r="N19" s="15" t="n"/>
-      <c r="O19" s="16" t="n"/>
-      <c r="P19" s="20" t="inlineStr">
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
+      <c r="M20" s="16" t="n"/>
+      <c r="N20" s="16" t="n"/>
+      <c r="O20" s="17" t="n"/>
+      <c r="P20" s="21" t="inlineStr">
         <is>
           <t>玩具廠</t>
         </is>
       </c>
-      <c r="Q19" s="16" t="n"/>
-    </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="Q20" s="17" t="n"/>
+    </row>
+    <row r="21" ht="95" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>M6
 1/15（五）</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>量產出廠</t>
         </is>
       </c>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>最後驗貨合格，包裝出貨</t>
         </is>
       </c>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="19" t="inlineStr">
+      <c r="F21" s="16" t="n"/>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="17" t="n"/>
+      <c r="I21" s="20" t="inlineStr">
         <is>
           <t>① 出貨前最後驗貨（抽檢）合格
 ② 包裝、裝箱、出貨，附每隻的序號清單
@@ -1222,119 +1273,119 @@
 ④ 三個 App 公開上架；客服聯絡方式和保修條款上線</t>
         </is>
       </c>
-      <c r="J20" s="15" t="n"/>
-      <c r="K20" s="15" t="n"/>
-      <c r="L20" s="15" t="n"/>
-      <c r="M20" s="15" t="n"/>
-      <c r="N20" s="15" t="n"/>
-      <c r="O20" s="16" t="n"/>
-      <c r="P20" s="20" t="inlineStr">
+      <c r="J21" s="16" t="n"/>
+      <c r="K21" s="16" t="n"/>
+      <c r="L21" s="16" t="n"/>
+      <c r="M21" s="16" t="n"/>
+      <c r="N21" s="16" t="n"/>
+      <c r="O21" s="17" t="n"/>
+      <c r="P21" s="21" t="inlineStr">
         <is>
           <t>玩具廠
 我方</t>
         </is>
       </c>
-      <c r="Q20" s="16" t="n"/>
-    </row>
-    <row r="21" ht="61" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="Q21" s="17" t="n"/>
+    </row>
+    <row r="22" ht="61" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>M7
 1/29（五）</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>送達客戶</t>
         </is>
       </c>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>全部送到客戶手上，開始使用</t>
         </is>
       </c>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="15" t="n"/>
-      <c r="H21" s="16" t="n"/>
-      <c r="I21" s="19" t="inlineStr">
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="17" t="n"/>
+      <c r="I22" s="20" t="inlineStr">
         <is>
           <t>① 全部簽收
 ② 首兩週每天檢查：對話成功率、回應速度、故障報告；問題 48 小時內處理</t>
         </is>
       </c>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="15" t="n"/>
-      <c r="L21" s="15" t="n"/>
-      <c r="M21" s="15" t="n"/>
-      <c r="N21" s="15" t="n"/>
-      <c r="O21" s="16" t="n"/>
-      <c r="P21" s="20" t="inlineStr">
+      <c r="J22" s="16" t="n"/>
+      <c r="K22" s="16" t="n"/>
+      <c r="L22" s="16" t="n"/>
+      <c r="M22" s="16" t="n"/>
+      <c r="N22" s="16" t="n"/>
+      <c r="O22" s="17" t="n"/>
+      <c r="P22" s="21" t="inlineStr">
         <is>
           <t>我方</t>
         </is>
       </c>
-      <c r="Q21" s="16" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="Q22" s="17" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>三、需要老闆知道的事</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>1. 客戶外觀簽樣最遲 11/13。晚一週簽，出廠就晚一週；過了 1/15 會拖到新年後（2 月底或 3 月）。</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="21" t="inlineStr">
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>2. 自家 AI Buddy 要不要在 1/15 一起出貨、出多少，最遲 11/27 要決定；要出貨的話，外觀也要在 11/13 前定。</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>3. 馬會和政協青年聯會要用自己的名義開 Apple／Google 開發者帳號（需時 1–3 週），App 才能以他們的品牌上架，請盡早向客戶提出。</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="21" t="inlineStr">
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
         <is>
           <t>4. 三個品牌各自一套獨立系統，客戶資料互不相通；程式只有一份，所以維護工作不會變成三倍。</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>每週的詳細進度在 project-schedule.xlsx，任務細項和測試記錄在 production-readiness.xlsx。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="55">
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="I14:O14"/>
+  <mergeCells count="60">
+    <mergeCell ref="A30:Q30"/>
     <mergeCell ref="I17:O17"/>
     <mergeCell ref="P20:Q20"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E16:H16"/>
-    <mergeCell ref="A24:Q24"/>
     <mergeCell ref="K9:O9"/>
     <mergeCell ref="I20:O20"/>
     <mergeCell ref="N6:Q6"/>
-    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="K10:N10"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="I19:O19"/>
+    <mergeCell ref="E22:H22"/>
     <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P22:Q22"/>
     <mergeCell ref="K8:M8"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E18:H18"/>
@@ -1345,17 +1396,19 @@
     <mergeCell ref="I15:O15"/>
     <mergeCell ref="A25:Q25"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="D10:G10"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E14:H14"/>
     <mergeCell ref="P17:Q17"/>
     <mergeCell ref="E17:H17"/>
     <mergeCell ref="A27:Q27"/>
     <mergeCell ref="A3:Q3"/>
     <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A12:Q12"/>
     <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="E20:H20"/>
     <mergeCell ref="A26:Q26"/>
     <mergeCell ref="A2:Q2"/>
@@ -1364,24 +1417,27 @@
     <mergeCell ref="E19:H19"/>
     <mergeCell ref="P19:Q19"/>
     <mergeCell ref="B16:D16"/>
+    <mergeCell ref="O10:Q10"/>
     <mergeCell ref="P18:Q18"/>
     <mergeCell ref="E9:H9"/>
+    <mergeCell ref="I22:O22"/>
+    <mergeCell ref="I10:J10"/>
     <mergeCell ref="P15:Q15"/>
     <mergeCell ref="I18:O18"/>
-    <mergeCell ref="A29:Q29"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="I21:O21"/>
     <mergeCell ref="G8:I8"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="E15:H15"/>
-    <mergeCell ref="P14:Q14"/>
     <mergeCell ref="B21:D21"/>
+    <mergeCell ref="A28:Q28"/>
     <mergeCell ref="I9:J9"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="22" min="0" max="16383" man="1"/>
+    <brk id="23" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>